<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-14 06:24:14
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>86.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-4.65</v>
+        <v>-0.22</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T14:27:06+08:00</t>
+          <t>2026-09-14T14:24:09+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-10.69</v>
+        <v>-10.89</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T14:27:07+08:00</t>
+          <t>2026-09-14T14:24:10+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>86.09999999999999</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-4.65</v>
+        <v>-0.22</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -929,13 +929,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-10.69</v>
+        <v>-10.89</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         <v>2.48</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-13.37</v>
+        <v>-13.66</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-10.69</v>
+        <v>-10.89</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -957,7 +957,9 @@
       <c r="L3" s="2" t="n">
         <v>-3.86</v>
       </c>
-      <c r="M3" s="2" t="n"/>
+      <c r="M3" s="2" t="n">
+        <v>-10.89</v>
+      </c>
       <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="n"/>
@@ -1167,16 +1169,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>21311936512</v>
+        <v>22302038016</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>29.385664</v>
+        <v>30.750853</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>13.601895</v>
+        <v>14.233808</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.758466</v>
+        <v>2.8866177</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1231,7 +1233,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T14:27:06+08:00</t>
+          <t>2026-09-14T14:24:09+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1257,16 +1259,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>431258566656</v>
+        <v>430302363648</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>43.91431</v>
+        <v>43.75304</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.383179</v>
+        <v>27.322462</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.4586363</v>
+        <v>4.4487505</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1293,7 +1295,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.54</v>
+        <v>20.57</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1321,7 +1323,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-11T14:27:07+08:00</t>
+          <t>2026-09-14T14:24:10+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-15 06:24:13
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.22</v>
+        <v>-1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T14:24:09+08:00</t>
+          <t>2026-09-15T14:24:08+08:00</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>900</v>
+        <v>914</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-10.89</v>
+        <v>-9.5</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>T11-15中段</t>
+          <t>T16-20成熟</t>
         </is>
       </c>
       <c r="J3" s="2" t="n"/>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T14:24:10+08:00</t>
+          <t>2026-09-15T14:24:09+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.22</v>
+        <v>-1</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -929,17 +929,17 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>900</v>
+        <v>914</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-10.89</v>
+        <v>-9.5</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>T11-15中段</t>
+          <t>T16-20成熟</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -995,10 +995,10 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1168,21 +1168,11 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>22302038016</v>
-      </c>
-      <c r="E2" s="2" t="n">
-        <v>30.750853</v>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>14.233808</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>2.8866177</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>13.2</v>
-      </c>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n">
         <v>29.62</v>
       </c>
@@ -1204,12 +1194,8 @@
       <c r="O2" s="2" t="n">
         <v>390.37</v>
       </c>
-      <c r="P2" s="2" t="n">
-        <v>2.93</v>
-      </c>
-      <c r="Q2" s="2" t="n">
-        <v>6.33</v>
-      </c>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n">
         <v>5080089000</v>
       </c>
@@ -1233,7 +1219,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T14:24:09+08:00</t>
+          <t>2026-09-15T14:24:08+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1258,21 +1244,11 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
-        <v>430302363648</v>
-      </c>
-      <c r="E3" s="2" t="n">
-        <v>43.75304</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>27.322462</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>4.4487505</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>10.85</v>
-      </c>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="n">
         <v>20.64</v>
       </c>
@@ -1294,12 +1270,8 @@
       <c r="O3" s="2" t="n">
         <v>159.5</v>
       </c>
-      <c r="P3" s="2" t="n">
-        <v>20.57</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>32.93993</v>
-      </c>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n">
         <v>15214310000</v>
       </c>
@@ -1323,7 +1295,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-14T14:24:10+08:00</t>
+          <t>2026-09-15T14:24:09+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-16 06:22:29
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>89.40000000000001</v>
+        <v>94.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1</v>
+        <v>4.98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T14:24:08+08:00</t>
+          <t>2026-09-16T14:22:25+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>914</v>
+        <v>937</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-9.5</v>
+        <v>-7.23</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T14:24:09+08:00</t>
+          <t>2026-09-16T14:22:25+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>89.40000000000001</v>
+        <v>94.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1</v>
+        <v>4.98</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -929,13 +929,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>914</v>
+        <v>937</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-9.5</v>
+        <v>-7.23</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -995,10 +995,10 @@
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1168,11 +1168,21 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
+      <c r="D2" s="2" t="n">
+        <v>23465408512</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>32.35495</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>14.976304</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>3.0371962</v>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>13.2</v>
+      </c>
       <c r="I2" s="2" t="n">
         <v>29.62</v>
       </c>
@@ -1194,8 +1204,12 @@
       <c r="O2" s="2" t="n">
         <v>390.37</v>
       </c>
-      <c r="P2" s="2" t="n"/>
-      <c r="Q2" s="2" t="n"/>
+      <c r="P2" s="2" t="n">
+        <v>2.93</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>6.33</v>
+      </c>
       <c r="R2" s="2" t="n">
         <v>5080089000</v>
       </c>
@@ -1219,7 +1233,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T14:24:08+08:00</t>
+          <t>2026-09-16T14:22:25+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1244,11 +1258,21 @@
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="D3" s="2" t="n">
+        <v>447992561664</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45.573933</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>28.445719</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>4.6316433</v>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>10.85</v>
+      </c>
       <c r="I3" s="2" t="n">
         <v>20.64</v>
       </c>
@@ -1270,8 +1294,12 @@
       <c r="O3" s="2" t="n">
         <v>159.5</v>
       </c>
-      <c r="P3" s="2" t="n"/>
-      <c r="Q3" s="2" t="n"/>
+      <c r="P3" s="2" t="n">
+        <v>20.56</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>32.93993</v>
+      </c>
       <c r="R3" s="2" t="n">
         <v>15214310000</v>
       </c>
@@ -1295,7 +1323,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-15T14:24:09+08:00</t>
+          <t>2026-09-16T14:22:25+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-17 06:26:44
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>94.8</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4.98</v>
+        <v>2.55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T14:22:25+08:00</t>
+          <t>2026-09-17T14:26:38+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>937</v>
+        <v>912</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-7.23</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T14:22:25+08:00</t>
+          <t>2026-09-17T14:26:39+08:00</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="15" customWidth="1" min="22" max="22"/>
     <col width="10" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>94.8</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4.98</v>
+        <v>2.55</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -893,9 +893,15 @@
       <c r="M2" s="2" t="n">
         <v>-1.11</v>
       </c>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
-      <c r="P2" s="2" t="n"/>
+      <c r="N2" s="2" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="O2" s="2" t="n">
+        <v>15.73</v>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>-7.2</v>
+      </c>
       <c r="Q2" s="2" t="n"/>
       <c r="R2" s="2" t="n"/>
       <c r="S2" s="2" t="b">
@@ -909,7 +915,7 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>T20_Completed</t>
         </is>
       </c>
       <c r="W2" s="2" t="n"/>
@@ -929,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>937</v>
+        <v>912</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-7.23</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1169,16 +1175,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23465408512</v>
+        <v>22920851456</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.35495</v>
+        <v>31.604094</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.976304</v>
+        <v>14.628752</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0371962</v>
+        <v>2.9667127</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1233,7 +1239,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T14:22:25+08:00</t>
+          <t>2026-09-17T14:26:38+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1259,16 +1265,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>447992561664</v>
+        <v>436039712768</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45.573933</v>
+        <v>44.444443</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28.445719</v>
+        <v>27.686762</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.6316433</v>
+        <v>4.508067</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1295,7 +1301,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.56</v>
+        <v>20.52</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.93993</v>
@@ -1323,7 +1329,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-16T14:22:25+08:00</t>
+          <t>2026-09-17T14:26:39+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-18 06:24:34
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -619,11 +619,11 @@
         <v>2.55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>T16-20成熟</t>
+          <t>T20後績效驗收</t>
         </is>
       </c>
       <c r="J2" s="2" t="n"/>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T14:26:38+08:00</t>
+          <t>2026-09-18T14:24:28+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>912</v>
+        <v>944</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-6.53</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T14:26:39+08:00</t>
+          <t>2026-09-18T14:24:29+08:00</t>
         </is>
       </c>
     </row>
@@ -868,11 +868,11 @@
         <v>2.55</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>T16-20成熟</t>
+          <t>T20後績效驗收</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>912</v>
+        <v>944</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-6.53</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T14:26:38+08:00</t>
+          <t>2026-09-18T14:24:28+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1265,16 +1265,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>436039712768</v>
+        <v>451339354112</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>44.444443</v>
+        <v>46.0039</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.686762</v>
+        <v>29.095535</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.508067</v>
+        <v>4.666245</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1304,7 +1304,7 @@
         <v>20.52</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>32.93993</v>
+        <v>32.44484</v>
       </c>
       <c r="R3" s="2" t="n">
         <v>15214310000</v>
@@ -1329,7 +1329,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-17T14:26:39+08:00</t>
+          <t>2026-09-18T14:24:29+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-21 06:25:49
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.59999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.55</v>
+        <v>3.32</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T14:24:28+08:00</t>
+          <t>2026-09-21T14:25:42+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>944</v>
+        <v>931</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-6.53</v>
+        <v>-7.82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T14:24:29+08:00</t>
+          <t>2026-09-21T14:25:43+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.59999999999999</v>
+        <v>93.3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.55</v>
+        <v>3.32</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>944</v>
+        <v>931</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-6.53</v>
+        <v>-7.82</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -966,9 +966,15 @@
       <c r="M3" s="2" t="n">
         <v>-10.89</v>
       </c>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
-      <c r="P3" s="2" t="n"/>
+      <c r="N3" s="2" t="n">
+        <v>-7.82</v>
+      </c>
+      <c r="O3" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>-13.66</v>
+      </c>
       <c r="Q3" s="2" t="n"/>
       <c r="R3" s="2" t="n"/>
       <c r="S3" s="2" t="b">
@@ -978,7 +984,7 @@
       <c r="U3" s="2" t="n"/>
       <c r="V3" s="2" t="inlineStr">
         <is>
-          <t>Tracking</t>
+          <t>T20_Completed</t>
         </is>
       </c>
       <c r="W3" s="2" t="n"/>
@@ -1175,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22920851456</v>
+        <v>23094120448</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.604094</v>
+        <v>31.843004</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.628752</v>
+        <v>14.739337</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9667127</v>
+        <v>2.9891393</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1239,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T14:24:28+08:00</t>
+          <t>2026-09-21T14:25:42+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1265,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>451339354112</v>
+        <v>445123887104</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.0039</v>
+        <v>45.238094</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.095535</v>
+        <v>28.694857</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.666245</v>
+        <v>4.601985</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1301,7 +1307,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.52</v>
+        <v>20.58</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>32.44484</v>
@@ -1329,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-18T14:24:29+08:00</t>
+          <t>2026-09-21T14:25:43+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-22 06:25:32
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>93.3</v>
+        <v>93.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.32</v>
+        <v>3.54</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:25:42+08:00</t>
+          <t>2026-09-22T14:25:27+08:00</t>
         </is>
       </c>
     </row>
@@ -664,17 +664,17 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>931</v>
+        <v>971</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-7.82</v>
+        <v>-3.86</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>T16-20成熟</t>
+          <t>T20後績效驗收</t>
         </is>
       </c>
       <c r="J3" s="2" t="n"/>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:25:43+08:00</t>
+          <t>2026-09-22T14:25:28+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>93.3</v>
+        <v>93.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>3.32</v>
+        <v>3.54</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,17 +935,17 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>931</v>
+        <v>971</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-7.82</v>
+        <v>-3.86</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>T16-20成熟</t>
+          <t>T20後績效驗收</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -1181,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23094120448</v>
+        <v>23143624704</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.843004</v>
+        <v>31.911263</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.739337</v>
+        <v>14.770932</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9891393</v>
+        <v>2.9955468</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:25:42+08:00</t>
+          <t>2026-09-22T14:25:27+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>445123887104</v>
+        <v>464248438784</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45.238094</v>
+        <v>47.18173</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28.694857</v>
+        <v>28.216604</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.601985</v>
+        <v>4.7997074</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1310,7 +1310,7 @@
         <v>20.58</v>
       </c>
       <c r="Q3" s="2" t="n">
-        <v>32.44484</v>
+        <v>34.41236</v>
       </c>
       <c r="R3" s="2" t="n">
         <v>15214310000</v>
@@ -1335,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-21T14:25:43+08:00</t>
+          <t>2026-09-22T14:25:28+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-23 06:25:22
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>93.5</v>
+        <v>95.7</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.54</v>
+        <v>5.98</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T14:25:27+08:00</t>
+          <t>2026-09-23T14:25:16+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>971</v>
+        <v>950</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-3.86</v>
+        <v>-5.94</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T14:25:28+08:00</t>
+          <t>2026-09-23T14:25:16+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>93.5</v>
+        <v>95.7</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>3.54</v>
+        <v>5.98</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>971</v>
+        <v>950</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-3.86</v>
+        <v>-5.94</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1181,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23143624704</v>
+        <v>23688181760</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.911263</v>
+        <v>32.662113</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.770932</v>
+        <v>15.118484</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9955468</v>
+        <v>3.0660303</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T14:25:27+08:00</t>
+          <t>2026-09-23T14:25:16+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>464248438784</v>
+        <v>454208028672</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>47.18173</v>
+        <v>46.1389</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28.216604</v>
+        <v>27.60636</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.7997074</v>
+        <v>4.6959033</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1307,7 +1307,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.58</v>
+        <v>20.59</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1335,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22T14:25:28+08:00</t>
+          <t>2026-09-23T14:25:16+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-24 06:25:25
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>95.7</v>
+        <v>94.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5.98</v>
+        <v>4.65</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T14:25:16+08:00</t>
+          <t>2026-09-24T14:25:19+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-5.94</v>
+        <v>-6.14</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T14:25:16+08:00</t>
+          <t>2026-09-24T14:25:19+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>95.7</v>
+        <v>94.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>5.98</v>
+        <v>4.65</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-5.94</v>
+        <v>-6.14</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1181,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23688181760</v>
+        <v>23391150080</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.662113</v>
+        <v>32.25256</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.118484</v>
+        <v>14.92891</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0660303</v>
+        <v>3.0275848</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T14:25:16+08:00</t>
+          <t>2026-09-24T14:25:19+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>454208028672</v>
+        <v>453251825664</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.1389</v>
+        <v>46.19883</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.60636</v>
+        <v>27.54824</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.6959033</v>
+        <v>4.686017</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1307,7 +1307,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.59</v>
+        <v>20.52</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1335,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-23T14:25:16+08:00</t>
+          <t>2026-09-24T14:25:19+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-29 06:24:50
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$Q$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Performance'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fundamentals'!$A$1:$Z$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Archive'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>94.5</v>
+        <v>95.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4.65</v>
+        <v>6.09</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T14:25:19+08:00</t>
+          <t>2026-09-29T14:24:46+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-6.14</v>
+        <v>-6.44</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T14:25:19+08:00</t>
+          <t>2026-09-29T14:24:46+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>94.5</v>
+        <v>95.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4.65</v>
+        <v>6.09</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>948</v>
+        <v>945</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-6.14</v>
+        <v>-6.44</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1181,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23391150080</v>
+        <v>23712933888</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.25256</v>
+        <v>32.696247</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.92891</v>
+        <v>15.134282</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0275848</v>
+        <v>3.0692341</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T14:25:19+08:00</t>
+          <t>2026-09-29T14:24:46+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>453251825664</v>
+        <v>451817472000</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>46.19883</v>
+        <v>45.940693</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.54824</v>
+        <v>27.461063</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.686017</v>
+        <v>4.671188</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1307,7 +1307,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.52</v>
+        <v>20.57</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1335,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24T14:25:19+08:00</t>
+          <t>2026-09-29T14:24:46+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -1356,16 +1356,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1422,34 +1422,14 @@
           <t>台半</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:08:26Z</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>TSM Stock Falls To Two-Month Low Amid Semiconductor Sell-Off Despite Wave Of Price Target Hikes</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Stocktwits</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>TSMC’s stock traded below $400 for the first time since May, marking the seventh straight day of losses for the shares.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>https://stocktwits.com/news-articles/markets/equity/tsm-stock-two-month-low-semiconductor-selloff-price-target-hikes/cZZ7laVR7MG</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>no_news</t>
         </is>
       </c>
     </row>
@@ -1464,123 +1444,19 @@
           <t>環球晶</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T18:29:34Z</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Direxion Daily Semiconductor Bull 3X ETF Explodes</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Motley Fool</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>If you like semiconductor stocks, you're going to love what's happening at Direxion today.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fool.com/investing/2026/07/09/direxion-daily-semiconductor-bull-3x-etf-explodes/</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>6488</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>環球晶</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T18:11:00Z</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Micron Unveils $250 Billion Spending Plan. BofA Says Buy.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Barrons.com</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Micron stock has dropped from levels of more than $1,200 and BofA analysts say there's a chance to buy at a discount.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.barrons.com/articles/micron-stock-price-analyst-buy-spending-19ebab1a?siteid=yhoof2&amp;yptr=yahoo</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>6488</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>環球晶</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T13:57:18Z</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>GlobalFoundries Shares Rise After Micron Expands U.S. Semiconductor Supply Chain Investment (GFS)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>InvestorsHub</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Micron Investment Boosts Confidence in U. S.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>https://investorshub.advfn.com/market-news/article/31596/globalfoundries-shares-rise-after-micron-expands-u-s-semiconductor-supply-chain-investment-gfs</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>no_news</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-09-30 06:24:07
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>95.8</v>
+        <v>96</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6.09</v>
+        <v>6.31</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:24:46+08:00</t>
+          <t>2026-09-30T14:24:03+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +664,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>945</v>
+        <v>1035</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-6.44</v>
+        <v>2.48</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +686,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:24:46+08:00</t>
+          <t>2026-09-30T14:24:03+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +862,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>95.8</v>
+        <v>96</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6.09</v>
+        <v>6.31</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +935,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>945</v>
+        <v>1035</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-6.44</v>
+        <v>2.48</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1181,16 +1181,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23712933888</v>
+        <v>23762440192</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.696247</v>
+        <v>32.764503</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.134282</v>
+        <v>15.165877</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0692341</v>
+        <v>3.0756416</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1245,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:24:46+08:00</t>
+          <t>2026-09-30T14:24:03+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1271,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>451817472000</v>
+        <v>494847721472</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>45.940693</v>
+        <v>50.242718</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27.461063</v>
+        <v>30.076403</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.671188</v>
+        <v>5.116063</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1307,7 +1307,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.57</v>
+        <v>20.6</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1335,7 +1335,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29T14:24:46+08:00</t>
+          <t>2026-09-30T14:24:03+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-01 06:27:00
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$Q$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Performance'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fundamentals'!$A$1:$Z$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Archive'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,8 +495,8 @@
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
     <col width="11" customWidth="1" min="16" max="16"/>
     <col width="27" customWidth="1" min="17" max="17"/>
   </cols>
@@ -613,29 +613,49 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>96</v>
+        <v>97.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6.31</v>
+        <v>7.97</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
           <t>T20後績效驗收</t>
         </is>
       </c>
-      <c r="J2" s="2" t="n"/>
-      <c r="K2" s="2" t="n"/>
-      <c r="L2" s="2" t="n"/>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
+      <c r="J2" s="2" t="n">
+        <v>71.05</v>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Weak</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>14.5%</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T14:24:03+08:00</t>
+          <t>2026-10-01T14:26:54+08:00</t>
         </is>
       </c>
     </row>
@@ -664,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1035</v>
+        <v>1085</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2.48</v>
+        <v>7.43</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -686,7 +706,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T14:24:03+08:00</t>
+          <t>2026-10-01T14:26:55+08:00</t>
         </is>
       </c>
     </row>
@@ -862,13 +882,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>96</v>
+        <v>97.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6.31</v>
+        <v>7.97</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -935,13 +955,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1035</v>
+        <v>1085</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>2.48</v>
+        <v>7.43</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -949,7 +969,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>2.48</v>
+        <v>12.38</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>-13.66</v>
@@ -1181,16 +1201,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23762440192</v>
+        <v>24133728256</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.764503</v>
+        <v>33.27645</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.165877</v>
+        <v>15.402843</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0756416</v>
+        <v>3.1236985</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1245,7 +1265,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T14:24:03+08:00</t>
+          <t>2026-10-01T14:26:54+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1271,16 +1291,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>494847721472</v>
+        <v>518753386496</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>50.242718</v>
+        <v>52.669903</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>30.076403</v>
+        <v>31.529367</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.116063</v>
+        <v>5.363216</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1335,7 +1355,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-09-30T14:24:03+08:00</t>
+          <t>2026-10-01T14:26:55+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -1356,16 +1376,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1422,14 +1442,34 @@
           <t>台半</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-17T14:08:26Z</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>TSM Stock Falls To Two-Month Low Amid Semiconductor Sell-Off Despite Wave Of Price Target Hikes</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Stocktwits</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>TSMC’s stock traded below $400 for the first time since May, marking the seventh straight day of losses for the shares.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://stocktwits.com/news-articles/markets/equity/tsm-stock-two-month-low-semiconductor-selloff-price-target-hikes/cZZ7laVR7MG</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>no_news</t>
+          <t>ok</t>
         </is>
       </c>
     </row>
@@ -1444,19 +1484,123 @@
           <t>環球晶</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T18:29:34Z</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Direxion Daily Semiconductor Bull 3X ETF Explodes</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Motley Fool</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>If you like semiconductor stocks, you're going to love what's happening at Direxion today.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fool.com/investing/2026/07/09/direxion-daily-semiconductor-bull-3x-etf-explodes/</t>
+        </is>
+      </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>no_news</t>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>6488</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>環球晶</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T18:11:00Z</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Micron Unveils $250 Billion Spending Plan. BofA Says Buy.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Barrons.com</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Micron stock has dropped from levels of more than $1,200 and BofA analysts say there's a chance to buy at a discount.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.barrons.com/articles/micron-stock-price-analyst-buy-spending-19ebab1a?siteid=yhoof2&amp;yptr=yahoo</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>6488</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>環球晶</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09T13:57:18Z</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>GlobalFoundries Shares Rise After Micron Expands U.S. Semiconductor Supply Chain Investment (GFS)</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>InvestorsHub</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Micron Investment Boosts Confidence in U. S.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://investorshub.advfn.com/market-news/article/31596/globalfoundries-shares-rise-after-micron-expands-u-s-semiconductor-supply-chain-investment-gfs</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>ok</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:H5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-02 06:25:21
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Overview'!$A$1:$Q$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Performance'!$A$1:$W$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Fundamentals'!$A$1:$Z$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'News'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Archive'!$A$1:$I$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>97.5</v>
+        <v>102</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>7.97</v>
+        <v>12.96</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -627,19 +627,19 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>71.05</v>
+        <v>78.34</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>54.6</v>
+        <v>69.44</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Weak</t>
+          <t>Moderate</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>14.5%</t>
+          <t>19.1%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:26:54+08:00</t>
+          <t>2026-10-02T14:25:15+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1085</v>
+        <v>1190</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>7.43</v>
+        <v>17.82</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:26:55+08:00</t>
+          <t>2026-10-02T14:25:16+08:00</t>
         </is>
       </c>
     </row>
@@ -882,13 +882,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>97.5</v>
+        <v>102</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.97</v>
+        <v>12.96</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -955,13 +955,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1085</v>
+        <v>1190</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>7.43</v>
+        <v>17.82</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12.38</v>
+        <v>17.82</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>-13.66</v>
@@ -1201,16 +1201,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24133728256</v>
+        <v>25247592448</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>33.27645</v>
+        <v>34.812286</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.402843</v>
+        <v>16.113745</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.1236985</v>
+        <v>3.2678692</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1265,7 +1265,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:26:54+08:00</t>
+          <t>2026-10-02T14:25:15+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1291,16 +1291,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>518753386496</v>
+        <v>568955305984</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>52.669903</v>
+        <v>58.020477</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>31.529367</v>
+        <v>34.580597</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.363216</v>
+        <v>5.8822365</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1327,7 +1327,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.6</v>
+        <v>20.51</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1355,7 +1355,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-01T14:26:55+08:00</t>
+          <t>2026-10-02T14:25:16+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">
@@ -1376,16 +1376,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="48" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1442,34 +1442,14 @@
           <t>台半</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-17T14:08:26Z</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>TSM Stock Falls To Two-Month Low Amid Semiconductor Sell-Off Despite Wave Of Price Target Hikes</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Stocktwits</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>TSMC’s stock traded below $400 for the first time since May, marking the seventh straight day of losses for the shares.</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>https://stocktwits.com/news-articles/markets/equity/tsm-stock-two-month-low-semiconductor-selloff-price-target-hikes/cZZ7laVR7MG</t>
-        </is>
-      </c>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>no_news</t>
         </is>
       </c>
     </row>
@@ -1484,123 +1464,19 @@
           <t>環球晶</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T18:29:34Z</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Direxion Daily Semiconductor Bull 3X ETF Explodes</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Motley Fool</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>If you like semiconductor stocks, you're going to love what's happening at Direxion today.</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>https://www.fool.com/investing/2026/07/09/direxion-daily-semiconductor-bull-3x-etf-explodes/</t>
-        </is>
-      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+      <c r="F3" s="2" t="n"/>
+      <c r="G3" s="2" t="n"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>6488</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>環球晶</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T18:11:00Z</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Micron Unveils $250 Billion Spending Plan. BofA Says Buy.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Barrons.com</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Micron stock has dropped from levels of more than $1,200 and BofA analysts say there's a chance to buy at a discount.</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>https://www.barrons.com/articles/micron-stock-price-analyst-buy-spending-19ebab1a?siteid=yhoof2&amp;yptr=yahoo</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>6488</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>環球晶</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>2026-07-09T13:57:18Z</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>GlobalFoundries Shares Rise After Micron Expands U.S. Semiconductor Supply Chain Investment (GFS)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>InvestorsHub</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Micron Investment Boosts Confidence in U. S.</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>https://investorshub.advfn.com/market-news/article/31596/globalfoundries-shares-rise-after-micron-expands-u-s-semiconductor-supply-chain-investment-gfs</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>ok</t>
+          <t>no_news</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:H3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-05 06:24:53
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>102</v>
+        <v>105.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>12.96</v>
+        <v>16.83</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:25:15+08:00</t>
+          <t>2026-10-05T14:24:47+08:00</t>
         </is>
       </c>
     </row>
@@ -684,29 +684,49 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1190</v>
+        <v>1180</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>17.82</v>
+        <v>16.83</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>T20後績效驗收</t>
         </is>
       </c>
-      <c r="J3" s="2" t="n"/>
-      <c r="K3" s="2" t="n"/>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
+      <c r="J3" s="2" t="n">
+        <v>73.56999999999999</v>
+      </c>
+      <c r="K3" s="2" t="n">
+        <v>63.92</v>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>≥20%</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>BullTrend</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>unclassified</t>
+        </is>
+      </c>
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:25:16+08:00</t>
+          <t>2026-10-05T14:24:47+08:00</t>
         </is>
       </c>
     </row>
@@ -882,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>102</v>
+        <v>105.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>12.96</v>
+        <v>16.83</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -896,7 +916,7 @@
         </is>
       </c>
       <c r="H2" s="2" t="n">
-        <v>15.73</v>
+        <v>24.03</v>
       </c>
       <c r="I2" s="2" t="n">
         <v>-7.2</v>
@@ -955,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1190</v>
+        <v>1180</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>17.82</v>
+        <v>16.83</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -969,7 +989,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>17.82</v>
+        <v>22.28</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>-13.66</v>
@@ -1030,7 +1050,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1201,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>25247592448</v>
+        <v>26113931264</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>34.812286</v>
+        <v>35.64189</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>16.113745</v>
+        <v>16.666666</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.2678692</v>
+        <v>3.380002</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1237,7 +1257,7 @@
         <v>390.37</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>2.93</v>
+        <v>2.96</v>
       </c>
       <c r="Q2" s="2" t="n">
         <v>6.33</v>
@@ -1265,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:25:15+08:00</t>
+          <t>2026-10-05T14:24:47+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1291,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>568955305984</v>
+        <v>564174192640</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>58.020477</v>
+        <v>57.365097</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>34.580597</v>
+        <v>34.290005</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.8822365</v>
+        <v>5.832806</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1327,7 +1347,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.51</v>
+        <v>20.57</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1355,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02T14:25:16+08:00</t>
+          <t>2026-10-05T14:24:47+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-06 06:24:40
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>105.5</v>
+        <v>100.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>16.83</v>
+        <v>11.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -627,10 +627,10 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>78.34</v>
+        <v>72.63</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>69.44</v>
+        <v>60.64</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T14:24:47+08:00</t>
+          <t>2026-10-06T14:24:33+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1180</v>
+        <v>1205</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>16.83</v>
+        <v>19.31</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>73.56999999999999</v>
+        <v>75.66</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>63.92</v>
+        <v>66.20999999999999</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T14:24:47+08:00</t>
+          <t>2026-10-06T14:24:34+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>105.5</v>
+        <v>100.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>16.83</v>
+        <v>11.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1180</v>
+        <v>1205</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>16.83</v>
+        <v>19.31</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="H3" s="2" t="n">
-        <v>22.28</v>
+        <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
         <v>-13.66</v>
@@ -1050,7 +1050,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>26113931264</v>
+        <v>24876304384</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>35.64189</v>
+        <v>33.9527</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>16.666666</v>
+        <v>15.876778</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.380002</v>
+        <v>3.2198124</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T14:24:47+08:00</t>
+          <t>2026-10-06T14:24:33+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>564174192640</v>
+        <v>576127041536</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>57.365097</v>
+        <v>58.58046</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>34.290005</v>
+        <v>35.016487</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.832806</v>
+        <v>5.9563823</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-05T14:24:47+08:00</t>
+          <t>2026-10-06T14:24:34+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-07 06:28:05
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>100.5</v>
+        <v>104.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>11.3</v>
+        <v>15.73</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -627,10 +627,10 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>72.63</v>
+        <v>79.23</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>60.64</v>
+        <v>68.29000000000001</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
@@ -639,7 +639,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>19.1%</t>
+          <t>≥20%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:24:33+08:00</t>
+          <t>2026-10-07T14:28:00+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1205</v>
+        <v>1215</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>19.31</v>
+        <v>20.3</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -698,10 +698,10 @@
         </is>
       </c>
       <c r="J3" s="2" t="n">
-        <v>75.66</v>
+        <v>74.75</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>66.20999999999999</v>
+        <v>60.89</v>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:24:34+08:00</t>
+          <t>2026-10-07T14:28:00+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>100.5</v>
+        <v>104.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>11.3</v>
+        <v>15.73</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1205</v>
+        <v>1215</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>19.31</v>
+        <v>20.3</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24876304384</v>
+        <v>25866405888</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>33.9527</v>
+        <v>35.304054</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.876778</v>
+        <v>16.50869</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.2198124</v>
+        <v>3.347964</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:24:33+08:00</t>
+          <t>2026-10-07T14:28:00+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>576127041536</v>
+        <v>580908154880</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>58.58046</v>
+        <v>59.066605</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>35.016487</v>
+        <v>35.30708</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.9563823</v>
+        <v>6.005813</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-06T14:24:34+08:00</t>
+          <t>2026-10-07T14:28:00+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-12 06:24:33
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>104.5</v>
+        <v>100.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>15.73</v>
+        <v>11.3</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -627,19 +627,19 @@
         </is>
       </c>
       <c r="J2" s="2" t="n">
-        <v>79.23</v>
+        <v>74.84999999999999</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>68.29000000000001</v>
+        <v>44.32</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Moderate</t>
+          <t>Weak</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>≥20%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:28:00+08:00</t>
+          <t>2026-10-12T14:24:26+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1215</v>
+        <v>1115</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>20.3</v>
+        <v>10.4</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:28:00+08:00</t>
+          <t>2026-10-12T14:24:27+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>104.5</v>
+        <v>100.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>15.73</v>
+        <v>11.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1215</v>
+        <v>1115</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>20.3</v>
+        <v>10.4</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>25866405888</v>
+        <v>24876304384</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>35.304054</v>
+        <v>33.9527</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>16.50869</v>
+        <v>15.876778</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.347964</v>
+        <v>3.2198124</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:28:00+08:00</t>
+          <t>2026-10-12T14:24:26+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>580908154880</v>
+        <v>533096792064</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>59.066605</v>
+        <v>54.205154</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>35.30708</v>
+        <v>32.401146</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>6.005813</v>
+        <v>5.5115075</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-07T14:28:00+08:00</t>
+          <t>2026-10-12T14:24:27+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-13 06:22:24
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,10 +613,10 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>100.5</v>
+        <v>95.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>11.3</v>
+        <v>6.09</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>34</v>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T14:24:26+08:00</t>
+          <t>2026-10-13T14:22:18+08:00</t>
         </is>
       </c>
     </row>
@@ -684,10 +684,10 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1115</v>
+        <v>1015</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>10.4</v>
+        <v>0.5</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>32</v>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T14:24:27+08:00</t>
+          <t>2026-10-13T14:22:18+08:00</t>
         </is>
       </c>
     </row>
@@ -902,10 +902,10 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>100.5</v>
+        <v>95.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>11.3</v>
+        <v>6.09</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>34</v>
@@ -975,10 +975,10 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1115</v>
+        <v>1015</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>10.4</v>
+        <v>0.5</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>32</v>
@@ -995,7 +995,7 @@
         <v>-13.66</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-10.89</v>
+        <v>-16.46</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24876304384</v>
+        <v>23712933888</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>33.9527</v>
+        <v>32.364864</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.876778</v>
+        <v>15.134282</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.2198124</v>
+        <v>3.0692341</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T14:24:26+08:00</t>
+          <t>2026-10-13T14:22:18+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>533096792064</v>
+        <v>485285429248</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>54.205154</v>
+        <v>48.681053</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>32.401146</v>
+        <v>29.495214</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.5115075</v>
+        <v>5.017202</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1347,7 +1347,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.57</v>
+        <v>20.85</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-12T14:24:27+08:00</t>
+          <t>2026-10-13T14:22:18+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-14 06:23:58
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>95.8</v>
+        <v>97.2</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>6.09</v>
+        <v>7.64</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T14:22:18+08:00</t>
+          <t>2026-10-14T14:23:51+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.5</v>
+        <v>0.99</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T14:22:18+08:00</t>
+          <t>2026-10-14T14:23:52+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>95.8</v>
+        <v>97.2</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6.09</v>
+        <v>7.64</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1015</v>
+        <v>1020</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.5</v>
+        <v>0.99</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23712933888</v>
+        <v>24059469824</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.364864</v>
+        <v>32.837837</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.134282</v>
+        <v>15.35545</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0692341</v>
+        <v>3.114087</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T14:22:18+08:00</t>
+          <t>2026-10-14T14:23:51+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>485285429248</v>
+        <v>487676018688</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>48.681053</v>
+        <v>49.586777</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.495214</v>
+        <v>29.640512</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.017202</v>
+        <v>5.0419173</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1347,7 +1347,7 @@
         <v>159.5</v>
       </c>
       <c r="P3" s="2" t="n">
-        <v>20.85</v>
+        <v>20.57</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>34.41236</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-13T14:22:18+08:00</t>
+          <t>2026-10-14T14:23:52+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-15 06:23:20
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>97.2</v>
+        <v>92.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>7.64</v>
+        <v>2.44</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T14:23:51+08:00</t>
+          <t>2026-10-15T14:23:12+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>1020</v>
+        <v>923</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.99</v>
+        <v>-8.609999999999999</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T14:23:52+08:00</t>
+          <t>2026-10-15T14:23:13+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>97.2</v>
+        <v>92.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>7.64</v>
+        <v>2.44</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-10.87</v>
+        <v>-12.32</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>1020</v>
+        <v>923</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.99</v>
+        <v>-8.609999999999999</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         <v>-13.66</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-16.46</v>
+        <v>-24.03</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>24059469824</v>
+        <v>22896099328</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.837837</v>
+        <v>31.25</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.35545</v>
+        <v>14.612954</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.114087</v>
+        <v>2.9635088</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T14:23:51+08:00</t>
+          <t>2026-10-15T14:23:12+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>487676018688</v>
+        <v>441298976768</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>49.586777</v>
+        <v>44.871174</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>29.640512</v>
+        <v>26.821758</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>5.0419173</v>
+        <v>4.562441</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-14T14:23:52+08:00</t>
+          <t>2026-10-15T14:23:13+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-16 06:21:55
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.5</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.44</v>
+        <v>2.55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T14:23:12+08:00</t>
+          <t>2026-10-16T14:21:49+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>923</v>
+        <v>902</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-8.609999999999999</v>
+        <v>-10.69</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T14:23:13+08:00</t>
+          <t>2026-10-16T14:21:50+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.5</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.44</v>
+        <v>2.55</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>923</v>
+        <v>902</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-8.609999999999999</v>
+        <v>-10.69</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         <v>-13.66</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-24.03</v>
+        <v>-25.76</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22896099328</v>
+        <v>22920851456</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.25</v>
+        <v>32.83688</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>14.612954</v>
+        <v>15.721562</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9635088</v>
+        <v>2.9667127</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1257,10 +1257,10 @@
         <v>390.37</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>2.96</v>
+        <v>2.82</v>
       </c>
       <c r="Q2" s="2" t="n">
-        <v>6.33</v>
+        <v>5.89</v>
       </c>
       <c r="R2" s="2" t="n">
         <v>5080089000</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T14:23:12+08:00</t>
+          <t>2026-10-16T14:21:49+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>441298976768</v>
+        <v>431258566656</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>44.871174</v>
+        <v>43.85027</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26.821758</v>
+        <v>26.211512</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.562441</v>
+        <v>4.4586363</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-15T14:23:13+08:00</t>
+          <t>2026-10-16T14:21:50+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-19 06:24:34
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.59999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.55</v>
+        <v>1.22</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T14:21:49+08:00</t>
+          <t>2026-10-19T14:24:26+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>902</v>
+        <v>882</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-10.69</v>
+        <v>-12.67</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T14:21:50+08:00</t>
+          <t>2026-10-19T14:24:28+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.59999999999999</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.55</v>
+        <v>1.22</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-12.32</v>
+        <v>-13.36</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>902</v>
+        <v>882</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-10.69</v>
+        <v>-12.67</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
         <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-13.66</v>
+        <v>-17.03</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-25.76</v>
+        <v>-27.41</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22920851456</v>
+        <v>22623821824</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>32.83688</v>
+        <v>30.878378</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.721562</v>
+        <v>15.517827</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9667127</v>
+        <v>2.9282672</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1257,7 +1257,7 @@
         <v>390.37</v>
       </c>
       <c r="P2" s="2" t="n">
-        <v>2.82</v>
+        <v>2.96</v>
       </c>
       <c r="Q2" s="2" t="n">
         <v>5.89</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T14:21:49+08:00</t>
+          <t>2026-10-19T14:24:26+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>431258566656</v>
+        <v>421696307200</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>43.85027</v>
+        <v>42.87798</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>26.211512</v>
+        <v>25.630325</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.4586363</v>
+        <v>4.3597755</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16T14:21:50+08:00</t>
+          <t>2026-10-19T14:24:28+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-20 06:24:40
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>1.22</v>
+        <v>0.22</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:24:26+08:00</t>
+          <t>2026-10-20T14:24:34+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>882</v>
+        <v>844</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-12.67</v>
+        <v>-16.44</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:24:28+08:00</t>
+          <t>2026-10-20T14:24:35+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>91.40000000000001</v>
+        <v>90.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1.22</v>
+        <v>0.22</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-13.36</v>
+        <v>-14.22</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>882</v>
+        <v>844</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-12.67</v>
+        <v>-16.44</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         <v>-17.03</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-27.41</v>
+        <v>-30.53</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22623821824</v>
+        <v>22401048576</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.878378</v>
+        <v>30.574324</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.517827</v>
+        <v>15.3650255</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9282672</v>
+        <v>2.899433</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:24:26+08:00</t>
+          <t>2026-10-20T14:24:34+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>421696307200</v>
+        <v>403527991296</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>42.87798</v>
+        <v>41.03063</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>25.630325</v>
+        <v>24.526072</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.3597755</v>
+        <v>4.1719394</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-19T14:24:28+08:00</t>
+          <t>2026-10-20T14:24:35+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-21 06:25:49
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>90.5</v>
+        <v>94</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.22</v>
+        <v>4.1</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T14:24:34+08:00</t>
+          <t>2026-10-21T14:25:43+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>844</v>
+        <v>880</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-16.44</v>
+        <v>-12.87</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T14:24:35+08:00</t>
+          <t>2026-10-21T14:25:44+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>90.5</v>
+        <v>94</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.22</v>
+        <v>4.1</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>844</v>
+        <v>880</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-16.44</v>
+        <v>-12.87</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22401048576</v>
+        <v>23267387392</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.574324</v>
+        <v>31.756756</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.3650255</v>
+        <v>15.959253</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.899433</v>
+        <v>3.0115657</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T14:24:34+08:00</t>
+          <t>2026-10-21T14:25:43+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>403527991296</v>
+        <v>420740071424</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>41.03063</v>
+        <v>42.78075</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>24.526072</v>
+        <v>25.572206</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.1719394</v>
+        <v>4.3498893</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-20T14:24:35+08:00</t>
+          <t>2026-10-21T14:25:44+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-22 06:23:56
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>94</v>
+        <v>88.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>4.1</v>
+        <v>-1.66</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T14:25:43+08:00</t>
+          <t>2026-10-22T14:23:50+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>880</v>
+        <v>826</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-12.87</v>
+        <v>-18.22</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T14:25:44+08:00</t>
+          <t>2026-10-22T14:23:51+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>94</v>
+        <v>88.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>4.1</v>
+        <v>-1.66</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-14.22</v>
+        <v>-15.83</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>880</v>
+        <v>826</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-12.87</v>
+        <v>-18.22</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
         <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-17.03</v>
+        <v>-19.31</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-30.53</v>
+        <v>-32.02</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>23267387392</v>
+        <v>21980256256</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.756756</v>
+        <v>30</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.959253</v>
+        <v>15.076402</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>3.0115657</v>
+        <v>2.8449686</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T14:25:43+08:00</t>
+          <t>2026-10-22T14:23:50+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>420740071424</v>
+        <v>394921934848</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>42.78075</v>
+        <v>40.155567</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>25.572206</v>
+        <v>24.003002</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.3498893</v>
+        <v>4.0829644</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-21T14:25:44+08:00</t>
+          <t>2026-10-22T14:23:51+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-22 07:07:01
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T14:23:50+08:00</t>
+          <t>2026-10-22T15:06:56+08:00</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T14:23:51+08:00</t>
+          <t>2026-10-22T15:06:56+08:00</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T14:23:50+08:00</t>
+          <t>2026-10-22T15:06:56+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T14:23:51+08:00</t>
+          <t>2026-10-22T15:06:56+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-27 06:24:11
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>88.8</v>
+        <v>89.5</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-1.66</v>
+        <v>-0.89</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T15:06:56+08:00</t>
+          <t>2026-10-27T14:24:03+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>826</v>
+        <v>814</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-18.22</v>
+        <v>-19.41</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T15:06:56+08:00</t>
+          <t>2026-10-27T14:24:04+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>88.8</v>
+        <v>89.5</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-1.66</v>
+        <v>-0.89</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>826</v>
+        <v>814</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-18.22</v>
+        <v>-19.41</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
         <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-19.31</v>
+        <v>-20.1</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-32.02</v>
+        <v>-33</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>21980256256</v>
+        <v>22153523200</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30</v>
+        <v>30.236486</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.076402</v>
+        <v>15.195247</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8449686</v>
+        <v>2.8673952</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T15:06:56+08:00</t>
+          <t>2026-10-27T14:24:03+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>394921934848</v>
+        <v>429884571648</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>40.155567</v>
+        <v>39.572193</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>24.003002</v>
+        <v>23.654291</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.0829644</v>
+        <v>4.023648</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-22T15:06:56+08:00</t>
+          <t>2026-10-27T14:24:04+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-28 06:24:39
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>89.5</v>
+        <v>92.3</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.89</v>
+        <v>2.21</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T14:24:03+08:00</t>
+          <t>2026-10-28T14:24:34+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>814</v>
+        <v>849</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-19.41</v>
+        <v>-15.94</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T14:24:04+08:00</t>
+          <t>2026-10-28T14:24:35+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>89.5</v>
+        <v>92.3</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.89</v>
+        <v>2.21</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>814</v>
+        <v>849</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-19.41</v>
+        <v>-15.94</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22153523200</v>
+        <v>22846595072</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.236486</v>
+        <v>31.182432</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.195247</v>
+        <v>15.6706295</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8673952</v>
+        <v>2.9571013</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T14:24:03+08:00</t>
+          <t>2026-10-28T14:24:34+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>429884571648</v>
+        <v>448368541696</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>39.572193</v>
+        <v>41.2737</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>23.654291</v>
+        <v>24.671368</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.023648</v>
+        <v>4.1966543</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-27T14:24:04+08:00</t>
+          <t>2026-10-28T14:24:35+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-29 06:24:14
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>92.3</v>
+        <v>89.8</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.21</v>
+        <v>-0.55</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:24:34+08:00</t>
+          <t>2026-10-29T14:24:08+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>849</v>
+        <v>814</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-15.94</v>
+        <v>-19.41</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:24:35+08:00</t>
+          <t>2026-10-29T14:24:09+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>92.3</v>
+        <v>89.8</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>2.21</v>
+        <v>-0.55</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>849</v>
+        <v>814</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-15.94</v>
+        <v>-19.41</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -992,7 +992,7 @@
         <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-20.1</v>
+        <v>-20.5</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>-33</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22846595072</v>
+        <v>22227781632</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>31.182432</v>
+        <v>30.33784</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.6706295</v>
+        <v>15.246181</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.9571013</v>
+        <v>2.8770065</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:24:34+08:00</t>
+          <t>2026-10-29T14:24:08+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>448368541696</v>
+        <v>429884571648</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>41.2737</v>
+        <v>39.572193</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>24.671368</v>
+        <v>23.654291</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.1966543</v>
+        <v>4.023648</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-28T14:24:35+08:00</t>
+          <t>2026-10-29T14:24:09+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>

<commit_message>
🤖 自動盤後數據、Swing BuyNow、Deep Recovery與績效稽核: 2026-10-30 06:24:29
</commit_message>
<xml_diff>
--- a/data/swing_user_watchlist_analysis.xlsx
+++ b/data/swing_user_watchlist_analysis.xlsx
@@ -613,13 +613,13 @@
         <v>90.3</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>89.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>-0.55</v>
+        <v>-4.87</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -655,7 +655,7 @@
       <c r="P2" s="2" t="n"/>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:24:08+08:00</t>
+          <t>2026-10-30T14:24:24+08:00</t>
         </is>
       </c>
     </row>
@@ -684,13 +684,13 @@
         <v>1010</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>814</v>
+        <v>756</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>-19.41</v>
+        <v>-25.15</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
       <c r="P3" s="2" t="n"/>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:24:09+08:00</t>
+          <t>2026-10-30T14:24:24+08:00</t>
         </is>
       </c>
     </row>
@@ -902,13 +902,13 @@
         <v>90.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>89.8</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>-0.55</v>
+        <v>-4.87</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
         <v>-7.2</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>-15.83</v>
+        <v>-18.58</v>
       </c>
       <c r="K2" s="2" t="n">
         <v>5.43</v>
@@ -975,13 +975,13 @@
         <v>1010</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>814</v>
+        <v>756</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>-19.41</v>
+        <v>-25.15</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -992,10 +992,10 @@
         <v>24.75</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>-20.5</v>
+        <v>-26.63</v>
       </c>
       <c r="J3" s="2" t="n">
-        <v>-33</v>
+        <v>-37.78</v>
       </c>
       <c r="K3" s="2" t="n">
         <v>-9.699999999999999</v>
@@ -1221,16 +1221,16 @@
         </is>
       </c>
       <c r="D2" s="2" t="n">
-        <v>22227781632</v>
+        <v>21262432256</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>30.33784</v>
+        <v>29.020271</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>15.246181</v>
+        <v>14.584042</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>2.8770065</v>
+        <v>2.7520585</v>
       </c>
       <c r="H2" s="2" t="n">
         <v>13.2</v>
@@ -1285,7 +1285,7 @@
       <c r="X2" s="2" t="n"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:24:08+08:00</t>
+          <t>2026-10-30T14:24:24+08:00</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">
@@ -1311,16 +1311,16 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>429884571648</v>
+        <v>399253962752</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>39.572193</v>
+        <v>36.752552</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>23.654291</v>
+        <v>21.96885</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>4.023648</v>
+        <v>3.7369504</v>
       </c>
       <c r="H3" s="2" t="n">
         <v>10.85</v>
@@ -1375,7 +1375,7 @@
       <c r="X3" s="2" t="n"/>
       <c r="Y3" s="2" t="inlineStr">
         <is>
-          <t>2026-10-29T14:24:09+08:00</t>
+          <t>2026-10-30T14:24:24+08:00</t>
         </is>
       </c>
       <c r="Z3" s="2" t="inlineStr">

</xml_diff>